<commit_message>
Turn 0001: Macleod of Bow Valley takes Calgary Centre
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XTWKXtPrL9rvaUy4BKDKHi
</commit_message>
<xml_diff>
--- a/outputs/Riding_Tracker.xlsx
+++ b/outputs/Riding_Tracker.xlsx
@@ -781,7 +781,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I144"/>
+  <dimension ref="A1:I145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4205,27 +4205,27 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Pereira</t>
+          <t>Macleod</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>David Pereira</t>
+          <t>Sir Alexander Donald Macleod</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>G2</t>
+          <t>G1</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Ville-Marie—Le Sud-Ouest—Île-des-Soeurs</t>
+          <t>Calgary Centre</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>QC</t>
+          <t>AB</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -4235,16 +4235,16 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>Viscount Pereira of Mount Royal</t>
-        </is>
-      </c>
-      <c r="H78" s="37" t="inlineStr">
-        <is>
-          <t>#283969</t>
+          <t>Viscount Macleod of Bow Valley</t>
+        </is>
+      </c>
+      <c r="H78" s="36" t="inlineStr">
+        <is>
+          <t>#A89169</t>
         </is>
       </c>
       <c r="I78" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="79">
@@ -4265,7 +4265,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Laurier—Sainte-Marie</t>
+          <t>Ville-Marie—Le Sud-Ouest—Île-des-Soeurs</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -4283,13 +4283,13 @@
           <t>Viscount Pereira of Mount Royal</t>
         </is>
       </c>
-      <c r="H79" s="38" t="inlineStr">
-        <is>
-          <t>#5566A0</t>
+      <c r="H79" s="37" t="inlineStr">
+        <is>
+          <t>#283969</t>
         </is>
       </c>
       <c r="I79" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="80">
@@ -4310,7 +4310,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Outremont</t>
+          <t>Laurier—Sainte-Marie</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -4334,7 +4334,7 @@
         </is>
       </c>
       <c r="I80" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="81">
@@ -4355,7 +4355,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Papineau</t>
+          <t>Outremont</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -4379,7 +4379,7 @@
         </is>
       </c>
       <c r="I81" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="82">
@@ -4400,7 +4400,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Mount Royal</t>
+          <t>Papineau</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -4424,7 +4424,7 @@
         </is>
       </c>
       <c r="I82" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="83">
@@ -4445,7 +4445,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Saint-Laurent</t>
+          <t>Mount Royal</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -4469,47 +4469,52 @@
         </is>
       </c>
       <c r="I83" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Polkinghorne</t>
+          <t>Pereira</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>David Pereira</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>G1</t>
+          <t>G2</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Columbia—Kootenay—Southern Rockies</t>
+          <t>Saint-Laurent</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>BC</t>
+          <t>QC</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>Baron</t>
+          <t>Viscount</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>Baron Polkinghorne of Kootenay</t>
-        </is>
-      </c>
-      <c r="H84" s="39" t="inlineStr">
-        <is>
-          <t>#2A4F5F</t>
+          <t>Viscount Pereira of Mount Royal</t>
+        </is>
+      </c>
+      <c r="H84" s="38" t="inlineStr">
+        <is>
+          <t>#5566A0</t>
         </is>
       </c>
       <c r="I84" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="85">
@@ -4525,7 +4530,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Similkameen—South Okanagan—West Kootenay</t>
+          <t>Columbia—Kootenay—Southern Rockies</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -4543,13 +4548,13 @@
           <t>Baron Polkinghorne of Kootenay</t>
         </is>
       </c>
-      <c r="H85" s="40" t="inlineStr">
-        <is>
-          <t>#5A7F8F</t>
+      <c r="H85" s="39" t="inlineStr">
+        <is>
+          <t>#2A4F5F</t>
         </is>
       </c>
       <c r="I85" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="86">
@@ -4565,7 +4570,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Vernon—Lake Country—Monashee</t>
+          <t>Similkameen—South Okanagan—West Kootenay</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -4589,52 +4594,47 @@
         </is>
       </c>
       <c r="I86" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Richard-Arseneau</t>
-        </is>
-      </c>
-      <c r="B87" t="inlineStr">
-        <is>
-          <t>Olivier Richard-Arseneau</t>
+          <t>Polkinghorne</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>G3</t>
+          <t>G1</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Acadie—Bathurst</t>
+          <t>Vernon—Lake Country—Monashee</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>NB</t>
+          <t>BC</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>Marquis</t>
+          <t>Baron</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>Marquis Richard-Arseneau de la Chaleur</t>
-        </is>
-      </c>
-      <c r="H87" s="41" t="inlineStr">
-        <is>
-          <t>#2D6E6B</t>
+          <t>Baron Polkinghorne of Kootenay</t>
+        </is>
+      </c>
+      <c r="H87" s="40" t="inlineStr">
+        <is>
+          <t>#5A7F8F</t>
         </is>
       </c>
       <c r="I87" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="88">
@@ -4655,12 +4655,12 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Gaspésie—Les Îles-de-la-Madeleine—Listuguj</t>
+          <t>Acadie—Bathurst</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>QC</t>
+          <t>NB</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -4673,13 +4673,13 @@
           <t>Marquis Richard-Arseneau de la Chaleur</t>
         </is>
       </c>
-      <c r="H88" s="42" t="inlineStr">
-        <is>
-          <t>#5E9490</t>
+      <c r="H88" s="41" t="inlineStr">
+        <is>
+          <t>#2D6E6B</t>
         </is>
       </c>
       <c r="I88" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="89">
@@ -4700,12 +4700,12 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Miramichi—Grand Lake</t>
+          <t>Gaspésie—Les Îles-de-la-Madeleine—Listuguj</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>NB</t>
+          <t>QC</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -4724,7 +4724,7 @@
         </is>
       </c>
       <c r="I89" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="90">
@@ -4745,7 +4745,7 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Madawaska—Restigouche</t>
+          <t>Miramichi—Grand Lake</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
@@ -4769,7 +4769,7 @@
         </is>
       </c>
       <c r="I90" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="91">
@@ -4790,12 +4790,12 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Rimouski—La Matapédia</t>
+          <t>Madawaska—Restigouche</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>QC</t>
+          <t>NB</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -4814,7 +4814,7 @@
         </is>
       </c>
       <c r="I91" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="92">
@@ -4835,12 +4835,12 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Beauséjour</t>
+          <t>Rimouski—La Matapédia</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>NB</t>
+          <t>QC</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
@@ -4859,7 +4859,7 @@
         </is>
       </c>
       <c r="I92" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="93">
@@ -4880,7 +4880,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Moncton—Dieppe</t>
+          <t>Beauséjour</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -4904,7 +4904,7 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="94">
@@ -4925,12 +4925,12 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Côte-du-Sud—Rivière-du-Loup—Kataskomiq—Témiscouata</t>
+          <t>Moncton—Dieppe</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>QC</t>
+          <t>NB</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
@@ -4949,7 +4949,7 @@
         </is>
       </c>
       <c r="I94" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="95">
@@ -4970,12 +4970,12 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Fredericton—Oromocto</t>
+          <t>Côte-du-Sud—Rivière-du-Loup—Kataskomiq—Témiscouata</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>NB</t>
+          <t>QC</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
@@ -4994,7 +4994,7 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="96">
@@ -5015,12 +5015,12 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Bellechasse—Les Etchemins—Lévis</t>
+          <t>Fredericton—Oromocto</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>QC</t>
+          <t>NB</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
@@ -5039,7 +5039,7 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="97">
@@ -5060,7 +5060,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Beauce</t>
+          <t>Bellechasse—Les Etchemins—Lévis</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -5084,7 +5084,7 @@
         </is>
       </c>
       <c r="I97" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="98">
@@ -5105,7 +5105,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Québec Centre</t>
+          <t>Beauce</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
@@ -5129,7 +5129,7 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="99">
@@ -5150,12 +5150,12 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Fundy Royal</t>
+          <t>Québec Centre</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>NB</t>
+          <t>QC</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
@@ -5174,7 +5174,7 @@
         </is>
       </c>
       <c r="I99" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="100">
@@ -5195,7 +5195,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Saint John—Kennebecasis</t>
+          <t>Fundy Royal</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
@@ -5219,7 +5219,7 @@
         </is>
       </c>
       <c r="I100" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="101">
@@ -5240,12 +5240,12 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Louis-Hébert</t>
+          <t>Saint John—Kennebecasis</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>QC</t>
+          <t>NB</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
@@ -5264,7 +5264,7 @@
         </is>
       </c>
       <c r="I101" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="102">
@@ -5285,7 +5285,7 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Portneuf—Jacques-Cartier</t>
+          <t>Louis-Hébert</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
@@ -5309,7 +5309,7 @@
         </is>
       </c>
       <c r="I102" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="103">
@@ -5330,7 +5330,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Charlesbourg—Haute-Saint-Charles</t>
+          <t>Portneuf—Jacques-Cartier</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
@@ -5354,52 +5354,52 @@
         </is>
       </c>
       <c r="I103" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Ross</t>
+          <t>Richard-Arseneau</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Alexander James Ross</t>
+          <t>Olivier Richard-Arseneau</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>G2</t>
+          <t>G3</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Selkirk—Interlake—Eastman</t>
+          <t>Charlesbourg—Haute-Saint-Charles</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>MB</t>
+          <t>QC</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>Baron</t>
+          <t>Marquis</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>Baron Ross of Assiniboia</t>
-        </is>
-      </c>
-      <c r="H104" s="43" t="inlineStr">
-        <is>
-          <t>#5B7F8A</t>
+          <t>Marquis Richard-Arseneau de la Chaleur</t>
+        </is>
+      </c>
+      <c r="H104" s="42" t="inlineStr">
+        <is>
+          <t>#5E9490</t>
         </is>
       </c>
       <c r="I104" t="n">
-        <v>1</v>
+        <v>17</v>
       </c>
     </row>
     <row r="105">
@@ -5420,7 +5420,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Kildonan—St. Paul</t>
+          <t>Selkirk—Interlake—Eastman</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -5438,13 +5438,13 @@
           <t>Baron Ross of Assiniboia</t>
         </is>
       </c>
-      <c r="H105" s="44" t="inlineStr">
-        <is>
-          <t>#7A9DAB</t>
+      <c r="H105" s="43" t="inlineStr">
+        <is>
+          <t>#5B7F8A</t>
         </is>
       </c>
       <c r="I105" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="106">
@@ -5465,7 +5465,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Elmwood—Transcona</t>
+          <t>Kildonan—St. Paul</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
@@ -5489,7 +5489,7 @@
         </is>
       </c>
       <c r="I106" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="107">
@@ -5510,7 +5510,7 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Provencher</t>
+          <t>Elmwood—Transcona</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
@@ -5534,18 +5534,18 @@
         </is>
       </c>
       <c r="I107" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Sinclair-McKay</t>
+          <t>Ross</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Isabelle Ruth McKay</t>
+          <t>Alexander James Ross</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -5555,31 +5555,31 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Regina—Wascana</t>
+          <t>Provencher</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>SK</t>
+          <t>MB</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>Countess</t>
+          <t>Baron</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>Countess Sinclair-McKay of Kinookimaw</t>
-        </is>
-      </c>
-      <c r="H108" s="45" t="inlineStr">
-        <is>
-          <t>#3A6B8F</t>
+          <t>Baron Ross of Assiniboia</t>
+        </is>
+      </c>
+      <c r="H108" s="44" t="inlineStr">
+        <is>
+          <t>#7A9DAB</t>
         </is>
       </c>
       <c r="I108" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="109">
@@ -5600,7 +5600,7 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Regina—Qu'Appelle</t>
+          <t>Regina—Wascana</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -5618,13 +5618,13 @@
           <t>Countess Sinclair-McKay of Kinookimaw</t>
         </is>
       </c>
-      <c r="H109" s="46" t="inlineStr">
-        <is>
-          <t>#6693B8</t>
+      <c r="H109" s="45" t="inlineStr">
+        <is>
+          <t>#3A6B8F</t>
         </is>
       </c>
       <c r="I109" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="110">
@@ -5645,7 +5645,7 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Yorkton—Melville</t>
+          <t>Regina—Qu'Appelle</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
@@ -5669,7 +5669,7 @@
         </is>
       </c>
       <c r="I110" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="111">
@@ -5690,7 +5690,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Souris—Moose Mountain</t>
+          <t>Yorkton—Melville</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -5714,7 +5714,7 @@
         </is>
       </c>
       <c r="I111" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="112">
@@ -5735,7 +5735,7 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Moose Jaw—Lake Centre—Lanigan</t>
+          <t>Souris—Moose Mountain</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -5759,18 +5759,18 @@
         </is>
       </c>
       <c r="I112" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Stanton-Greville</t>
+          <t>Sinclair-McKay</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Edmund Stanton-Greville</t>
+          <t>Isabelle Ruth McKay</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -5780,31 +5780,31 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Bay of Quinte</t>
+          <t>Moose Jaw—Lake Centre—Lanigan</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>SK</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>Viscount</t>
+          <t>Countess</t>
         </is>
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>Viscount Stanton-Greville of Adolphustown</t>
-        </is>
-      </c>
-      <c r="H113" s="47" t="inlineStr">
-        <is>
-          <t>#8B1A1A</t>
+          <t>Countess Sinclair-McKay of Kinookimaw</t>
+        </is>
+      </c>
+      <c r="H113" s="46" t="inlineStr">
+        <is>
+          <t>#6693B8</t>
         </is>
       </c>
       <c r="I113" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="114">
@@ -5825,7 +5825,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Kingston and the Islands</t>
+          <t>Bay of Quinte</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
@@ -5843,13 +5843,13 @@
           <t>Viscount Stanton-Greville of Adolphustown</t>
         </is>
       </c>
-      <c r="H114" s="48" t="inlineStr">
-        <is>
-          <t>#B65757</t>
+      <c r="H114" s="47" t="inlineStr">
+        <is>
+          <t>#8B1A1A</t>
         </is>
       </c>
       <c r="I114" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="115">
@@ -5870,7 +5870,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Hastings—Lennox and Addington—Tyendinaga</t>
+          <t>Kingston and the Islands</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -5894,7 +5894,7 @@
         </is>
       </c>
       <c r="I115" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="116">
@@ -5915,7 +5915,7 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Leeds—Grenville—Thousand Islands—Rideau Lakes</t>
+          <t>Hastings—Lennox and Addington—Tyendinaga</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
@@ -5939,7 +5939,7 @@
         </is>
       </c>
       <c r="I116" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="117">
@@ -5960,7 +5960,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Stormont—Dundas—Glengarry</t>
+          <t>Leeds—Grenville—Thousand Islands—Rideau Lakes</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
@@ -5984,7 +5984,7 @@
         </is>
       </c>
       <c r="I117" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="118">
@@ -6005,7 +6005,7 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Lanark—Frontenac</t>
+          <t>Stormont—Dundas—Glengarry</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
@@ -6029,7 +6029,7 @@
         </is>
       </c>
       <c r="I118" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="119">
@@ -6050,7 +6050,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Northumberland—Clarke</t>
+          <t>Lanark—Frontenac</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
@@ -6074,18 +6074,18 @@
         </is>
       </c>
       <c r="I119" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Tessier</t>
+          <t>Stanton-Greville</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Paul-Léonard Tessier</t>
+          <t>Edmund Stanton-Greville</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -6095,31 +6095,31 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Laurentides—Labelle</t>
+          <t>Northumberland—Clarke</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>QC</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>Baron</t>
+          <t>Viscount</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>Baron Tessier de Saint-Jérôme</t>
-        </is>
-      </c>
-      <c r="H120" s="49" t="inlineStr">
-        <is>
-          <t>#4B3A6B</t>
+          <t>Viscount Stanton-Greville of Adolphustown</t>
+        </is>
+      </c>
+      <c r="H120" s="48" t="inlineStr">
+        <is>
+          <t>#B65757</t>
         </is>
       </c>
       <c r="I120" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="121">
@@ -6140,7 +6140,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Joliette—Manawan</t>
+          <t>Laurentides—Labelle</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
@@ -6158,13 +6158,13 @@
           <t>Baron Tessier de Saint-Jérôme</t>
         </is>
       </c>
-      <c r="H121" s="50" t="inlineStr">
-        <is>
-          <t>#5D4270</t>
+      <c r="H121" s="49" t="inlineStr">
+        <is>
+          <t>#4B3A6B</t>
         </is>
       </c>
       <c r="I121" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="122">
@@ -6185,7 +6185,7 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Les Pays-d'en-Haut</t>
+          <t>Joliette—Manawan</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
@@ -6209,7 +6209,7 @@
         </is>
       </c>
       <c r="I122" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="123">
@@ -6230,7 +6230,7 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Pontiac—Kitigan Zibi</t>
+          <t>Les Pays-d'en-Haut</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
@@ -6254,33 +6254,33 @@
         </is>
       </c>
       <c r="I123" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Trondek</t>
+          <t>Tessier</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Charlie Sékt'ìnka' Trondek</t>
+          <t>Paul-Léonard Tessier</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>G1</t>
+          <t>G2</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Yukon</t>
+          <t>Pontiac—Kitigan Zibi</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>YT</t>
+          <t>QC</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
@@ -6290,57 +6290,57 @@
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>Baron Trondek of Dawson</t>
-        </is>
-      </c>
-      <c r="H124" s="51" t="inlineStr">
-        <is>
-          <t>#7A6332</t>
+          <t>Baron Tessier de Saint-Jérôme</t>
+        </is>
+      </c>
+      <c r="H124" s="50" t="inlineStr">
+        <is>
+          <t>#5D4270</t>
         </is>
       </c>
       <c r="I124" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Wallace</t>
+          <t>Trondek</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Alexander James Wallace</t>
+          <t>Charlie Sékt'ìnka' Trondek</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>G2</t>
+          <t>G1</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Toronto Centre</t>
+          <t>Yukon</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>YT</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>Viscount</t>
+          <t>Baron</t>
         </is>
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>Viscount Wallace of Rosedale</t>
-        </is>
-      </c>
-      <c r="H125" s="52" t="inlineStr">
-        <is>
-          <t>#A44A1F</t>
+          <t>Baron Trondek of Dawson</t>
+        </is>
+      </c>
+      <c r="H125" s="51" t="inlineStr">
+        <is>
+          <t>#7A6332</t>
         </is>
       </c>
       <c r="I125" t="n">
@@ -6365,7 +6365,7 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Spadina—Harbourfront</t>
+          <t>Toronto Centre</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
@@ -6383,13 +6383,13 @@
           <t>Viscount Wallace of Rosedale</t>
         </is>
       </c>
-      <c r="H126" s="53" t="inlineStr">
-        <is>
-          <t>#C27550</t>
+      <c r="H126" s="52" t="inlineStr">
+        <is>
+          <t>#A44A1F</t>
         </is>
       </c>
       <c r="I126" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="127">
@@ -6410,7 +6410,7 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Taiaiako'n—Parkdale—High Park</t>
+          <t>Spadina—Harbourfront</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
@@ -6434,7 +6434,7 @@
         </is>
       </c>
       <c r="I127" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="128">
@@ -6455,7 +6455,7 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>University—Rosedale</t>
+          <t>Taiaiako'n—Parkdale—High Park</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
@@ -6479,7 +6479,7 @@
         </is>
       </c>
       <c r="I128" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="129">
@@ -6500,7 +6500,7 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Toronto—Danforth</t>
+          <t>University—Rosedale</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
@@ -6524,7 +6524,7 @@
         </is>
       </c>
       <c r="I129" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="130">
@@ -6545,7 +6545,7 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Toronto—St. Paul's</t>
+          <t>Toronto—Danforth</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
@@ -6569,7 +6569,7 @@
         </is>
       </c>
       <c r="I130" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="131">
@@ -6590,7 +6590,7 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Don Valley West</t>
+          <t>Toronto—St. Paul's</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
@@ -6614,18 +6614,18 @@
         </is>
       </c>
       <c r="I131" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>Whitcombe</t>
+          <t>Wallace</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>Edwin Whitcombe</t>
+          <t>Alexander James Wallace</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -6635,7 +6635,7 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Parry Sound—Muskoka</t>
+          <t>Don Valley West</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
@@ -6650,16 +6650,16 @@
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>Viscount Whitcombe of Muskoka</t>
-        </is>
-      </c>
-      <c r="H132" s="54" t="inlineStr">
-        <is>
-          <t>#2E5E3A</t>
+          <t>Viscount Wallace of Rosedale</t>
+        </is>
+      </c>
+      <c r="H132" s="53" t="inlineStr">
+        <is>
+          <t>#C27550</t>
         </is>
       </c>
       <c r="I132" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="133">
@@ -6680,7 +6680,7 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Nipissing—Timiskaming</t>
+          <t>Parry Sound—Muskoka</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
@@ -6698,13 +6698,13 @@
           <t>Viscount Whitcombe of Muskoka</t>
         </is>
       </c>
-      <c r="H133" s="55" t="inlineStr">
-        <is>
-          <t>#4A7A55</t>
+      <c r="H133" s="54" t="inlineStr">
+        <is>
+          <t>#2E5E3A</t>
         </is>
       </c>
       <c r="I133" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="134">
@@ -6725,7 +6725,7 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Sudbury East—Manitoulin—Nickel Belt</t>
+          <t>Nipissing—Timiskaming</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
@@ -6749,7 +6749,7 @@
         </is>
       </c>
       <c r="I134" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="135">
@@ -6770,7 +6770,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Algonquin—Renfrew—Pembroke</t>
+          <t>Sudbury East—Manitoulin—Nickel Belt</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
@@ -6794,7 +6794,7 @@
         </is>
       </c>
       <c r="I135" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="136">
@@ -6815,7 +6815,7 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>Kapuskasing—Timmins—Mushkegowuk</t>
+          <t>Algonquin—Renfrew—Pembroke</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
@@ -6839,7 +6839,7 @@
         </is>
       </c>
       <c r="I136" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="137">
@@ -6860,7 +6860,7 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Thunder Bay—Superior North</t>
+          <t>Kapuskasing—Timmins—Mushkegowuk</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
@@ -6884,7 +6884,7 @@
         </is>
       </c>
       <c r="I137" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="138">
@@ -6905,7 +6905,7 @@
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>Sault Ste. Marie—Algoma</t>
+          <t>Thunder Bay—Superior North</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
@@ -6929,7 +6929,7 @@
         </is>
       </c>
       <c r="I138" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="139">
@@ -6950,12 +6950,12 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>Abitibi—Baie-James—Nunavik—Eeyou</t>
+          <t>Sault Ste. Marie—Algoma</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>QC</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
@@ -6974,7 +6974,7 @@
         </is>
       </c>
       <c r="I139" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="140">
@@ -6995,12 +6995,12 @@
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>Thunder Bay—Rainy River</t>
+          <t>Abitibi—Baie-James—Nunavik—Eeyou</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>QC</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
@@ -7019,7 +7019,7 @@
         </is>
       </c>
       <c r="I140" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="141">
@@ -7040,7 +7040,7 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>Sudbury</t>
+          <t>Thunder Bay—Rainy River</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
@@ -7064,18 +7064,18 @@
         </is>
       </c>
       <c r="I141" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>Wilmot-Hazen</t>
+          <t>Whitcombe</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>Sir Edward John Wilmot-Hazen Jr.</t>
+          <t>Edwin Whitcombe</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
@@ -7085,31 +7085,31 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>Saint John—St. Croix</t>
+          <t>Sudbury</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>NB</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>Baron</t>
+          <t>Viscount</t>
         </is>
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>Baron Wilmot-Hazen of Saint John</t>
-        </is>
-      </c>
-      <c r="H142" s="56" t="inlineStr">
-        <is>
-          <t>#4A3828</t>
+          <t>Viscount Whitcombe of Muskoka</t>
+        </is>
+      </c>
+      <c r="H142" s="55" t="inlineStr">
+        <is>
+          <t>#4A7A55</t>
         </is>
       </c>
       <c r="I142" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="143">
@@ -7130,7 +7130,7 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>Tobique—Mactaquac</t>
+          <t>Saint John—St. Croix</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
@@ -7148,57 +7148,102 @@
           <t>Baron Wilmot-Hazen of Saint John</t>
         </is>
       </c>
-      <c r="H143" s="57" t="inlineStr">
-        <is>
-          <t>#A88860</t>
+      <c r="H143" s="56" t="inlineStr">
+        <is>
+          <t>#4A3828</t>
         </is>
       </c>
       <c r="I143" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
+          <t>Wilmot-Hazen</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Sir Edward John Wilmot-Hazen Jr.</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>G2</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Tobique—Mactaquac</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>Baron</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>Baron Wilmot-Hazen of Saint John</t>
+        </is>
+      </c>
+      <c r="H144" s="57" t="inlineStr">
+        <is>
+          <t>#A88860</t>
+        </is>
+      </c>
+      <c r="I144" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
           <t>Wilson</t>
         </is>
       </c>
-      <c r="B144" t="inlineStr">
+      <c r="B145" t="inlineStr">
         <is>
           <t>Cairine Wilson</t>
         </is>
       </c>
-      <c r="C144" t="inlineStr">
+      <c r="C145" t="inlineStr">
         <is>
           <t>G1</t>
         </is>
       </c>
-      <c r="D144" t="inlineStr">
+      <c r="D145" t="inlineStr">
         <is>
           <t>Ottawa—Vanier—Gloucester</t>
         </is>
       </c>
-      <c r="E144" t="inlineStr">
+      <c r="E145" t="inlineStr">
         <is>
           <t>ON</t>
         </is>
       </c>
-      <c r="F144" t="inlineStr">
+      <c r="F145" t="inlineStr">
         <is>
           <t>Baroness</t>
         </is>
       </c>
-      <c r="G144" t="inlineStr">
+      <c r="G145" t="inlineStr">
         <is>
           <t>Baroness Wilson of Rockcliffe</t>
         </is>
       </c>
-      <c r="H144" s="58" t="inlineStr">
+      <c r="H145" s="58" t="inlineStr">
         <is>
           <t>#7B3F7B</t>
         </is>
       </c>
-      <c r="I144" t="n">
+      <c r="I145" t="n">
         <v>1</v>
       </c>
     </row>
@@ -8344,7 +8389,7 @@
         </is>
       </c>
       <c r="L22" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="23">
@@ -13766,7 +13811,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I41"/>
+  <dimension ref="A1:I42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -13777,7 +13822,7 @@
     <col width="39" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="27" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -15024,6 +15069,49 @@
       <c r="H41" t="inlineStr">
         <is>
           <t>2026-09-06T00:57:48+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="n">
+        <v>1</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>expansion</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>The Counting-House Made Freehold</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Macleod</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>turn</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>2026-09-06 03:26:49</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Calgary Centre came to the house the way most things came to Sir Alexander Donald Macleod: by ledger first, and ceremony long afterwards.
+The Bureau on Stephen Avenue had been a convenience when the house took its rooms there — somewhere for the Macleod Ranching Co. to keep its accounts nearer the railhead than Bow River allowed. It did not stay a convenience. Turner Valley Petroleum Holdings lodged its subscription books in the same building; the ranching company's freight contracts followed; and by the close of the season's reconciliation the greater part of the house's commercial life was being conducted from a street the house did not hold.
+Sir Alexander, who had taken his barony at sixty-seven and his viscountcy since, was not sentimental about the discovery. He had built outward from Bow River in the order a cattleman builds a fence: the home quarter first, then east, then south to Shepard, then the long line north to Yellowhead. Calgary Centre was the gap he had been riding around for years. He put the case in one sitting and, characteristically, on one page: the house already held the ground on three sides of its counting-house, and it was an absurdity to remain a tenant in the room where its money was counted.
+Lady Margaret's objection was not to the taking but to the manner of it. She had watched the Bow Valley house become, by degrees, a Calgary house that kept cattle, and thought the change deserved saying out loud rather than accomplishing by lease renewals. So it was said out loud. The instrument was read at Knox Presbyterian on a Sunday of hard light, before a congregation that contained both halves of the house's awkward politics: the Liberal commercial men who banked with the Bureau, and the cooperative farmers who sold through it and mistrusted it. The Viscount, a founding director of the summer exhibition and used to standing between those two rooms, read the ochre and dun of his colours into the record and made no speech.
+The letters that followed were brief and, in their way, telling. Lockhart of Waterton wrote from the south with the dryness of a neighbour who had first met the house at its investiture and had been watching its accounts ever since. From Kinookimaw, the Countess Sinclair-McKay sent a single line of congratulation that managed to be both warm and a reminder that prairie houses are counted by what they hold at the end, not by what they take in the middle. Both were filed. Neither was answered at length.
+What the acquisition did not settle was the succession of the work. Donald Alexander, thirty-one years his father's junior and still unconfirmed as operational heir, spent the week after the reading in the Stephen Avenue rooms, learning which of the two ledgers — cattle or petroleum — the house would be judged by. The Viscount, asked, declined to answer. The fence was finished. Who would ride it was another season's business.</t>
         </is>
       </c>
     </row>
@@ -15038,11 +15126,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
@@ -15060,6 +15148,21 @@
       <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Macleod's personal clock has no recovered year, so this expansion cannot be placed on the house's own clock. The director must set it before any Macleod event that needs a date.</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>open</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reconstruction: Macleod house block; clock resume policy
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XTWKXtPrL9rvaUy4BKDKHi
</commit_message>
<xml_diff>
--- a/outputs/Riding_Tracker.xlsx
+++ b/outputs/Riding_Tracker.xlsx
@@ -9,13 +9,14 @@
   <sheets>
     <sheet name="Riding Tracker" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Houses" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Successions" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Climate" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Relations" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Matrix" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Events" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Watch" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Handoff" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="House Blocks" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Successions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Climate" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Relations" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Matrix" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Events" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Watch" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Handoff" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -7252,6 +7253,36 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Key</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -7373,9 +7404,12 @@
           <t>G1</t>
         </is>
       </c>
+      <c r="J2" t="n">
+        <v>1867</v>
+      </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>personal clock begins 1867 at founding; personal year not recovered</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L2" t="n">
@@ -7428,9 +7462,12 @@
           <t>Rajesh Anand (eldest son, ~25 at founding)</t>
         </is>
       </c>
+      <c r="J3" t="n">
+        <v>1867</v>
+      </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>reset to personal 1867 at accession founding (bio ~70 at grant, b. 1898 Lahore); personal year not recovered</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L3" t="n">
@@ -7478,9 +7515,12 @@
           <t>Thomas Ashworth</t>
         </is>
       </c>
+      <c r="J4" t="n">
+        <v>1867</v>
+      </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>personal clock begins 1867 at founding; personal year not recovered</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L4" t="n">
@@ -7528,9 +7568,12 @@
           <t>not formally named</t>
         </is>
       </c>
+      <c r="J5" t="n">
+        <v>1867</v>
+      </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>reset to personal 1867 at accession Blaikie personal 1916; personal year not recovered</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L5" t="n">
@@ -7578,9 +7621,12 @@
           <t>Marie-Louise Boyer-Lavallée (heir-apparent-operational)</t>
         </is>
       </c>
+      <c r="J6" t="n">
+        <v>1867</v>
+      </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>personal clock begins 1867 at founding; personal year not recovered</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L6" t="n">
@@ -7628,9 +7674,12 @@
           <t>Giuseppe Calabrese (eldest son, ~30 at founding)</t>
         </is>
       </c>
+      <c r="J7" t="n">
+        <v>1867</v>
+      </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>reset to personal 1867 at accession founding (bio ~70 at grant, b. 1898 Reggio Calabria); personal year not recovered</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L7" t="n">
@@ -7678,9 +7727,12 @@
           <t>Suzanne Cardinal (heir-apparent, operational principal)</t>
         </is>
       </c>
+      <c r="J8" t="n">
+        <v>1867</v>
+      </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>personal clock begins 1867 at founding; personal year not recovered</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L8" t="n">
@@ -7733,9 +7785,12 @@
           <t>not formally named</t>
         </is>
       </c>
+      <c r="J9" t="n">
+        <v>1867</v>
+      </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>reset to personal 1867 at accession summer Delany personal 1910; personal year not recovered</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L9" t="n">
@@ -7773,9 +7828,12 @@
           <t>G1</t>
         </is>
       </c>
+      <c r="J10" t="n">
+        <v>1867</v>
+      </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>personal clock begins 1867 at founding; personal year not recovered</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L10" t="n">
@@ -7823,9 +7881,12 @@
           <t>G2</t>
         </is>
       </c>
+      <c r="J11" t="n">
+        <v>1867</v>
+      </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>reset to personal 1867 at accession 1918 (as recorded); personal year not recovered</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L11" t="n">
@@ -7873,9 +7934,12 @@
           <t>not formally named</t>
         </is>
       </c>
+      <c r="J12" t="n">
+        <v>1867</v>
+      </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>reset to personal 1867 at accession spring Galbraith personal 1908; personal year not recovered</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L12" t="n">
@@ -7928,9 +7992,12 @@
           <t>not formally named</t>
         </is>
       </c>
+      <c r="J13" t="n">
+        <v>1867</v>
+      </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>reset to personal 1867 at accession autumn Garland personal 1909; personal year not recovered</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L13" t="n">
@@ -7983,9 +8050,12 @@
           <t>not formally named</t>
         </is>
       </c>
+      <c r="J14" t="n">
+        <v>1867</v>
+      </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>reset to personal 1867 at accession spring Hall personal 1920; personal year not recovered</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L14" t="n">
@@ -8028,9 +8098,12 @@
           <t>G1</t>
         </is>
       </c>
+      <c r="J15" t="n">
+        <v>1867</v>
+      </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>personal clock begins 1867 at founding; personal year not recovered</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L15" t="n">
@@ -8073,9 +8146,12 @@
           <t>G1</t>
         </is>
       </c>
+      <c r="J16" t="n">
+        <v>1867</v>
+      </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>personal clock begins 1867 at founding; personal year not recovered</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L16" t="n">
@@ -8123,9 +8199,12 @@
           <t>not formally named</t>
         </is>
       </c>
+      <c r="J17" t="n">
+        <v>1867</v>
+      </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>reset to personal 1867 at accession spring Letendre personal 1909; personal year not recovered</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L17" t="n">
@@ -8178,9 +8257,12 @@
           <t>operational heir, unnamed</t>
         </is>
       </c>
+      <c r="J18" t="n">
+        <v>1867</v>
+      </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>personal clock begins 1867 at founding; personal year not recovered</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L18" t="n">
@@ -8223,9 +8305,12 @@
           <t>G2</t>
         </is>
       </c>
+      <c r="J19" t="n">
+        <v>1867</v>
+      </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>accession not recovered; personal year not recovered</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L19" t="n">
@@ -8278,9 +8363,12 @@
           <t>not formally named</t>
         </is>
       </c>
+      <c r="J20" t="n">
+        <v>1867</v>
+      </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>reset to personal 1867 at accession winter MacDonald personal 1901; personal year not recovered</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L20" t="n">
@@ -8328,9 +8416,12 @@
           <t>G2</t>
         </is>
       </c>
+      <c r="J21" t="n">
+        <v>1867</v>
+      </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>accession not recovered; personal year not recovered</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L21" t="n">
@@ -8383,9 +8474,12 @@
           <t>Donald Alexander Macleod (b. 1893), unconfirmed</t>
         </is>
       </c>
+      <c r="J22" t="n">
+        <v>1867</v>
+      </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>reset to personal 1867 at accession founding (bio 67 at grant, b. 1862); personal year not recovered</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L22" t="n">
@@ -8433,9 +8527,12 @@
           <t>G2</t>
         </is>
       </c>
+      <c r="J23" t="n">
+        <v>1867</v>
+      </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>accession not recovered; personal year not recovered</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L23" t="n">
@@ -8478,9 +8575,12 @@
           <t>G1</t>
         </is>
       </c>
+      <c r="J24" t="n">
+        <v>1867</v>
+      </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>personal clock begins 1867 at founding; personal year not recovered</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L24" t="n">
@@ -8528,9 +8628,12 @@
           <t>G3</t>
         </is>
       </c>
+      <c r="J25" t="n">
+        <v>1867</v>
+      </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>accession not recovered; personal year not recovered</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L25" t="n">
@@ -8583,9 +8686,12 @@
           <t>not formally named</t>
         </is>
       </c>
+      <c r="J26" t="n">
+        <v>1867</v>
+      </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>reset to personal 1867 at accession Ross personal 1922; personal year not recovered</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L26" t="n">
@@ -8638,9 +8744,12 @@
           <t>not formally named</t>
         </is>
       </c>
+      <c r="J27" t="n">
+        <v>1867</v>
+      </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>reset to personal 1867 at accession spring SinM personal 1920; personal year not recovered</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L27" t="n">
@@ -8693,9 +8802,12 @@
           <t>not formally named</t>
         </is>
       </c>
+      <c r="J28" t="n">
+        <v>1867</v>
+      </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>reset to personal 1867 at accession autumn SG personal 1910; personal year not recovered</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L28" t="n">
@@ -8743,9 +8855,12 @@
           <t>G2</t>
         </is>
       </c>
+      <c r="J29" t="n">
+        <v>1867</v>
+      </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>accession not recovered; personal year not recovered</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L29" t="n">
@@ -8793,9 +8908,12 @@
           <t>Joseph Sékt'ìnka' Trondek (eldest son, ~30 at founding)</t>
         </is>
       </c>
+      <c r="J30" t="n">
+        <v>1867</v>
+      </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>reset to personal 1867 at accession founding (bio ~70 at grant, b. ~1875 Tr'ochëk); personal year not recovered</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L30" t="n">
@@ -8848,9 +8966,12 @@
           <t>not formally named</t>
         </is>
       </c>
+      <c r="J31" t="n">
+        <v>1867</v>
+      </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>reset to personal 1867 at accession autumn Wallace personal 1909; personal year not recovered</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L31" t="n">
@@ -8898,9 +9019,12 @@
           <t>G2</t>
         </is>
       </c>
+      <c r="J32" t="n">
+        <v>1867</v>
+      </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>accession not recovered; personal year not recovered</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L32" t="n">
@@ -8953,9 +9077,12 @@
           <t>not formally named</t>
         </is>
       </c>
+      <c r="J33" t="n">
+        <v>1867</v>
+      </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>reset to personal 1867 at accession Wilmot-Hazen personal 1925; personal year not recovered</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L33" t="n">
@@ -9003,9 +9130,12 @@
           <t>G1</t>
         </is>
       </c>
+      <c r="J34" t="n">
+        <v>1867</v>
+      </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>personal clock begins 1867 at founding; personal year not recovered</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L34" t="n">
@@ -9053,9 +9183,12 @@
           <t>not formally named</t>
         </is>
       </c>
+      <c r="J35" t="n">
+        <v>1867</v>
+      </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>reset to personal 1867 at accession autumn Kilmartin personal 1923; personal year not recovered</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L35" t="n">
@@ -9083,9 +9216,12 @@
           <t>G2</t>
         </is>
       </c>
+      <c r="J36" t="n">
+        <v>1867</v>
+      </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>accession not recovered; personal year not recovered</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L36" t="n">
@@ -9098,6 +9234,224 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="27" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>House</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Macleod</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Sir Alexander Donald Macleod (G1), b. 1862 / biological 67 at founding grant Macleod personal 1867. Glengarry-Ontario-born; emigrated west 1882 with CPR construction wave; Cochrane Ranche Company apprenticeship late 1880s; founded Macleod Ranching Co. Bow Valley 1893; Turner Valley petroleum early investor 1914+; Knox Presbyterian Calgary senior elder; Calgary Stampede founding director 1912. Married Lady Margaret Macleod (née MacKenzie, b. 1868); five children.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>founding block 2026-04-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Macleod</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Current holder</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Sir Alexander Donald Macleod, Baron Macleod of Bow Valley (G1, founding grant Macleod personal 1867). [Rank since raised to Viscount; elevation event not recovered.]</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>founding block 2026-04-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Macleod</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Heir apparent</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>None formally named at grant. Eldest son Donald Alexander Macleod (b. 1893, biological ~36 at grant) natural operational heir but unconfirmed.</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>founding block 2026-04-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Macleod</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Holdings</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Bow River (Macleod Ranch — Bow Valley House at Cochrane + Macleod Ranching Co. + Turner Valley Petroleum Holdings + Bureau Calgary + Fondation Macleod — Knox Presbyterian Calgary + UFA Cooperative Education Endowment, founding grant Macleod personal 1867). Later: Calgary East, Calgary Shepard, Yellowhead (expansion records not recovered); Calgary Centre (turn 0001).</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>founding block 2026-04-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Macleod</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Economic position</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Founding grant capital $80,000. Macleod Ranching Co. as primary commercial entity (cattle + horse + Hereford-stock improvement; Calgary stockyards + CPR shipping partnerships); Turner Valley Royalties ~12% — first tracker engagement with Alberta petroleum sector; Fondation Macleod UFA Cooperative Education Endowment as first tracker UFA-cooperative endowment partnership. Liberal-Presbyterian-UFA cooperative cross-axis institutional reach distinguishes Macleod from Lockhart's Conservative-Loyalist Foothills positioning despite shared Alberta peer-house status.</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>founding block 2026-04-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Macleod</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Political position</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Liberal-aligned commercial; UFA-adjacent cooperative-agricultural sympathies; Knox Presbyterian senior-elder establishment positioning. Cross-axis Liberal-commercial + UFA-cooperative + Presbyterian-establishment signature. TAG: Mixed (Section 10).</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>founding block 2026-04-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Macleod</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Cultural position</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Glengarry-rooted Scots-Albertan; bridges Eastern Ontario Scots-Presbyterian roots with western prairie commercial-establishment positioning; Calgary Stampede founding director gives Macleod distinct populist-civic positioning beyond pure commercial elite. Lady Margaret cultural-family representative.</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>founding block 2026-04-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Macleod</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Personal clock</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Macleod personal 1867 (founding grant; clock starts here per Section 1 rule). Sir Alexander Donald biological 67; Lady Margaret biological 61; eldest son Donald Alexander biological ~36 (natural operational heir).</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>founding block 2026-04-25</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -10119,7 +10473,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -10729,7 +11083,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -11983,7 +12337,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -13805,7 +14159,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -13898,7 +14252,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-09-06T00:57:48+00:00</t>
+          <t>2026-09-06T03:36:41+00:00</t>
         </is>
       </c>
     </row>
@@ -13928,7 +14282,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-09-06T00:57:48+00:00</t>
+          <t>2026-09-06T03:36:41+00:00</t>
         </is>
       </c>
     </row>
@@ -13958,7 +14312,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-09-06T00:57:48+00:00</t>
+          <t>2026-09-06T03:36:41+00:00</t>
         </is>
       </c>
     </row>
@@ -13988,7 +14342,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-09-06T00:57:48+00:00</t>
+          <t>2026-09-06T03:36:41+00:00</t>
         </is>
       </c>
     </row>
@@ -14018,7 +14372,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-09-06T00:57:48+00:00</t>
+          <t>2026-09-06T03:36:41+00:00</t>
         </is>
       </c>
     </row>
@@ -14048,7 +14402,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-09-06T00:57:48+00:00</t>
+          <t>2026-09-06T03:36:41+00:00</t>
         </is>
       </c>
     </row>
@@ -14078,7 +14432,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-09-06T00:57:48+00:00</t>
+          <t>2026-09-06T03:36:41+00:00</t>
         </is>
       </c>
     </row>
@@ -14108,7 +14462,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-09-06T00:57:48+00:00</t>
+          <t>2026-09-06T03:36:41+00:00</t>
         </is>
       </c>
     </row>
@@ -14138,7 +14492,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-09-06T00:57:48+00:00</t>
+          <t>2026-09-06T03:36:41+00:00</t>
         </is>
       </c>
     </row>
@@ -14168,7 +14522,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-09-06T00:57:48+00:00</t>
+          <t>2026-09-06T03:36:41+00:00</t>
         </is>
       </c>
     </row>
@@ -14198,7 +14552,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-09-06T00:57:48+00:00</t>
+          <t>2026-09-06T03:36:41+00:00</t>
         </is>
       </c>
     </row>
@@ -14228,7 +14582,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-09-06T00:57:48+00:00</t>
+          <t>2026-09-06T03:36:41+00:00</t>
         </is>
       </c>
     </row>
@@ -14258,7 +14612,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-09-06T00:57:48+00:00</t>
+          <t>2026-09-06T03:36:41+00:00</t>
         </is>
       </c>
     </row>
@@ -14288,7 +14642,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-09-06T00:57:48+00:00</t>
+          <t>2026-09-06T03:36:41+00:00</t>
         </is>
       </c>
     </row>
@@ -14318,7 +14672,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026-09-06T00:57:48+00:00</t>
+          <t>2026-09-06T03:36:41+00:00</t>
         </is>
       </c>
     </row>
@@ -14348,7 +14702,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026-09-06T00:57:48+00:00</t>
+          <t>2026-09-06T03:36:41+00:00</t>
         </is>
       </c>
     </row>
@@ -14378,7 +14732,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026-09-06T00:57:48+00:00</t>
+          <t>2026-09-06T03:36:41+00:00</t>
         </is>
       </c>
     </row>
@@ -14408,7 +14762,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2026-09-06T00:57:48+00:00</t>
+          <t>2026-09-06T03:36:41+00:00</t>
         </is>
       </c>
     </row>
@@ -14438,7 +14792,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>2026-09-06T00:57:48+00:00</t>
+          <t>2026-09-06T03:36:41+00:00</t>
         </is>
       </c>
     </row>
@@ -14468,7 +14822,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>2026-09-06T00:57:48+00:00</t>
+          <t>2026-09-06T03:36:41+00:00</t>
         </is>
       </c>
     </row>
@@ -14498,7 +14852,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>2026-09-06T00:57:48+00:00</t>
+          <t>2026-09-06T03:36:41+00:00</t>
         </is>
       </c>
     </row>
@@ -14528,7 +14882,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>2026-09-06T00:57:48+00:00</t>
+          <t>2026-09-06T03:36:41+00:00</t>
         </is>
       </c>
     </row>
@@ -14558,7 +14912,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>2026-09-06T00:57:48+00:00</t>
+          <t>2026-09-06T03:36:41+00:00</t>
         </is>
       </c>
     </row>
@@ -14588,7 +14942,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>2026-09-06T00:57:48+00:00</t>
+          <t>2026-09-06T03:36:41+00:00</t>
         </is>
       </c>
     </row>
@@ -14618,7 +14972,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>2026-09-06T00:57:48+00:00</t>
+          <t>2026-09-06T03:36:41+00:00</t>
         </is>
       </c>
     </row>
@@ -14648,7 +15002,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>2026-09-06T00:57:48+00:00</t>
+          <t>2026-09-06T03:36:41+00:00</t>
         </is>
       </c>
     </row>
@@ -14678,7 +15032,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>2026-09-06T00:57:48+00:00</t>
+          <t>2026-09-06T03:36:41+00:00</t>
         </is>
       </c>
     </row>
@@ -14708,7 +15062,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>2026-09-06T00:57:48+00:00</t>
+          <t>2026-09-06T03:36:41+00:00</t>
         </is>
       </c>
     </row>
@@ -14738,7 +15092,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>2026-09-06T00:57:48+00:00</t>
+          <t>2026-09-06T03:36:41+00:00</t>
         </is>
       </c>
     </row>
@@ -14768,7 +15122,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>2026-09-06T00:57:48+00:00</t>
+          <t>2026-09-06T03:36:41+00:00</t>
         </is>
       </c>
     </row>
@@ -14798,7 +15152,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>2026-09-06T00:57:48+00:00</t>
+          <t>2026-09-06T03:36:41+00:00</t>
         </is>
       </c>
     </row>
@@ -14828,7 +15182,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>2026-09-06T00:57:48+00:00</t>
+          <t>2026-09-06T03:36:41+00:00</t>
         </is>
       </c>
     </row>
@@ -14858,7 +15212,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>2026-09-06T00:57:48+00:00</t>
+          <t>2026-09-06T03:36:41+00:00</t>
         </is>
       </c>
     </row>
@@ -14888,7 +15242,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>2026-09-06T00:57:48+00:00</t>
+          <t>2026-09-06T03:36:41+00:00</t>
         </is>
       </c>
     </row>
@@ -14918,7 +15272,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>2026-09-06T00:57:48+00:00</t>
+          <t>2026-09-06T03:36:41+00:00</t>
         </is>
       </c>
     </row>
@@ -14948,7 +15302,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>2026-09-06T00:57:48+00:00</t>
+          <t>2026-09-06T03:36:41+00:00</t>
         </is>
       </c>
     </row>
@@ -14978,7 +15332,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>2026-09-06T00:57:48+00:00</t>
+          <t>2026-09-06T03:36:41+00:00</t>
         </is>
       </c>
     </row>
@@ -15008,7 +15362,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>2026-09-06T00:57:48+00:00</t>
+          <t>2026-09-06T03:36:41+00:00</t>
         </is>
       </c>
     </row>
@@ -15038,7 +15392,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>2026-09-06T00:57:48+00:00</t>
+          <t>2026-09-06T03:36:41+00:00</t>
         </is>
       </c>
     </row>
@@ -15068,7 +15422,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>2026-09-06T00:57:48+00:00</t>
+          <t>2026-09-06T03:36:41+00:00</t>
         </is>
       </c>
     </row>
@@ -15101,7 +15455,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>2026-09-06 03:26:49</t>
+          <t>2026-09-06 03:36:41</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -15120,7 +15474,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -15169,34 +15523,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Key</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Text</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Housekeeping turn 0002; rebuild script; threshold tweak
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XTWKXtPrL9rvaUy4BKDKHi
</commit_message>
<xml_diff>
--- a/outputs/Riding_Tracker.xlsx
+++ b/outputs/Riding_Tracker.xlsx
@@ -14165,7 +14165,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I42"/>
+  <dimension ref="A1:I43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -14252,7 +14252,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-09-06T03:36:41+00:00</t>
+          <t>2026-09-06T03:38:14+00:00</t>
         </is>
       </c>
     </row>
@@ -14282,7 +14282,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-09-06T03:36:41+00:00</t>
+          <t>2026-09-06T03:38:14+00:00</t>
         </is>
       </c>
     </row>
@@ -14312,7 +14312,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-09-06T03:36:41+00:00</t>
+          <t>2026-09-06T03:38:14+00:00</t>
         </is>
       </c>
     </row>
@@ -14342,7 +14342,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-09-06T03:36:41+00:00</t>
+          <t>2026-09-06T03:38:14+00:00</t>
         </is>
       </c>
     </row>
@@ -14372,7 +14372,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-09-06T03:36:41+00:00</t>
+          <t>2026-09-06T03:38:14+00:00</t>
         </is>
       </c>
     </row>
@@ -14402,7 +14402,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-09-06T03:36:41+00:00</t>
+          <t>2026-09-06T03:38:14+00:00</t>
         </is>
       </c>
     </row>
@@ -14432,7 +14432,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-09-06T03:36:41+00:00</t>
+          <t>2026-09-06T03:38:14+00:00</t>
         </is>
       </c>
     </row>
@@ -14462,7 +14462,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-09-06T03:36:41+00:00</t>
+          <t>2026-09-06T03:38:14+00:00</t>
         </is>
       </c>
     </row>
@@ -14492,7 +14492,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-09-06T03:36:41+00:00</t>
+          <t>2026-09-06T03:38:14+00:00</t>
         </is>
       </c>
     </row>
@@ -14522,7 +14522,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-09-06T03:36:41+00:00</t>
+          <t>2026-09-06T03:38:14+00:00</t>
         </is>
       </c>
     </row>
@@ -14552,7 +14552,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-09-06T03:36:41+00:00</t>
+          <t>2026-09-06T03:38:14+00:00</t>
         </is>
       </c>
     </row>
@@ -14582,7 +14582,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-09-06T03:36:41+00:00</t>
+          <t>2026-09-06T03:38:14+00:00</t>
         </is>
       </c>
     </row>
@@ -14612,7 +14612,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-09-06T03:36:41+00:00</t>
+          <t>2026-09-06T03:38:14+00:00</t>
         </is>
       </c>
     </row>
@@ -14642,7 +14642,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-09-06T03:36:41+00:00</t>
+          <t>2026-09-06T03:38:14+00:00</t>
         </is>
       </c>
     </row>
@@ -14672,7 +14672,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026-09-06T03:36:41+00:00</t>
+          <t>2026-09-06T03:38:14+00:00</t>
         </is>
       </c>
     </row>
@@ -14702,7 +14702,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026-09-06T03:36:41+00:00</t>
+          <t>2026-09-06T03:38:14+00:00</t>
         </is>
       </c>
     </row>
@@ -14732,7 +14732,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026-09-06T03:36:41+00:00</t>
+          <t>2026-09-06T03:38:14+00:00</t>
         </is>
       </c>
     </row>
@@ -14762,7 +14762,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2026-09-06T03:36:41+00:00</t>
+          <t>2026-09-06T03:38:14+00:00</t>
         </is>
       </c>
     </row>
@@ -14792,7 +14792,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>2026-09-06T03:36:41+00:00</t>
+          <t>2026-09-06T03:38:14+00:00</t>
         </is>
       </c>
     </row>
@@ -14822,7 +14822,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>2026-09-06T03:36:41+00:00</t>
+          <t>2026-09-06T03:38:14+00:00</t>
         </is>
       </c>
     </row>
@@ -14852,7 +14852,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>2026-09-06T03:36:41+00:00</t>
+          <t>2026-09-06T03:38:14+00:00</t>
         </is>
       </c>
     </row>
@@ -14882,7 +14882,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>2026-09-06T03:36:41+00:00</t>
+          <t>2026-09-06T03:38:14+00:00</t>
         </is>
       </c>
     </row>
@@ -14912,7 +14912,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>2026-09-06T03:36:41+00:00</t>
+          <t>2026-09-06T03:38:14+00:00</t>
         </is>
       </c>
     </row>
@@ -14942,7 +14942,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>2026-09-06T03:36:41+00:00</t>
+          <t>2026-09-06T03:38:14+00:00</t>
         </is>
       </c>
     </row>
@@ -14972,7 +14972,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>2026-09-06T03:36:41+00:00</t>
+          <t>2026-09-06T03:38:14+00:00</t>
         </is>
       </c>
     </row>
@@ -15002,7 +15002,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>2026-09-06T03:36:41+00:00</t>
+          <t>2026-09-06T03:38:14+00:00</t>
         </is>
       </c>
     </row>
@@ -15032,7 +15032,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>2026-09-06T03:36:41+00:00</t>
+          <t>2026-09-06T03:38:14+00:00</t>
         </is>
       </c>
     </row>
@@ -15062,7 +15062,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>2026-09-06T03:36:41+00:00</t>
+          <t>2026-09-06T03:38:14+00:00</t>
         </is>
       </c>
     </row>
@@ -15092,7 +15092,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>2026-09-06T03:36:41+00:00</t>
+          <t>2026-09-06T03:38:14+00:00</t>
         </is>
       </c>
     </row>
@@ -15122,7 +15122,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>2026-09-06T03:36:41+00:00</t>
+          <t>2026-09-06T03:38:14+00:00</t>
         </is>
       </c>
     </row>
@@ -15152,7 +15152,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>2026-09-06T03:36:41+00:00</t>
+          <t>2026-09-06T03:38:14+00:00</t>
         </is>
       </c>
     </row>
@@ -15182,7 +15182,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>2026-09-06T03:36:41+00:00</t>
+          <t>2026-09-06T03:38:14+00:00</t>
         </is>
       </c>
     </row>
@@ -15212,7 +15212,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>2026-09-06T03:36:41+00:00</t>
+          <t>2026-09-06T03:38:14+00:00</t>
         </is>
       </c>
     </row>
@@ -15242,7 +15242,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>2026-09-06T03:36:41+00:00</t>
+          <t>2026-09-06T03:38:14+00:00</t>
         </is>
       </c>
     </row>
@@ -15272,7 +15272,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>2026-09-06T03:36:41+00:00</t>
+          <t>2026-09-06T03:38:14+00:00</t>
         </is>
       </c>
     </row>
@@ -15302,7 +15302,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>2026-09-06T03:36:41+00:00</t>
+          <t>2026-09-06T03:38:14+00:00</t>
         </is>
       </c>
     </row>
@@ -15332,7 +15332,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>2026-09-06T03:36:41+00:00</t>
+          <t>2026-09-06T03:38:14+00:00</t>
         </is>
       </c>
     </row>
@@ -15362,7 +15362,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>2026-09-06T03:36:41+00:00</t>
+          <t>2026-09-06T03:38:14+00:00</t>
         </is>
       </c>
     </row>
@@ -15392,7 +15392,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>2026-09-06T03:36:41+00:00</t>
+          <t>2026-09-06T03:38:14+00:00</t>
         </is>
       </c>
     </row>
@@ -15422,7 +15422,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>2026-09-06T03:36:41+00:00</t>
+          <t>2026-09-06T03:38:14+00:00</t>
         </is>
       </c>
     </row>
@@ -15455,7 +15455,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>2026-09-06 03:36:41</t>
+          <t>2026-09-06 03:38:14</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -15466,6 +15466,40 @@
 Lady Margaret's objection was not to the taking but to the manner of it. She had watched the Bow Valley house become, by degrees, a Calgary house that kept cattle, and thought the change deserved saying out loud rather than accomplishing by lease renewals. So it was said out loud. The instrument was read at Knox Presbyterian on a Sunday of hard light, before a congregation that contained both halves of the house's awkward politics: the Liberal commercial men who banked with the Bureau, and the cooperative farmers who sold through it and mistrusted it. The Viscount, a founding director of the summer exhibition and used to standing between those two rooms, read the ochre and dun of his colours into the record and made no speech.
 The letters that followed were brief and, in their way, telling. Lockhart of Waterton wrote from the south with the dryness of a neighbour who had first met the house at its investiture and had been watching its accounts ever since. From Kinookimaw, the Countess Sinclair-McKay sent a single line of congratulation that managed to be both warm and a reminder that prairie houses are counted by what they hold at the end, not by what they take in the middle. Both were filed. Neither was answered at length.
 What the acquisition did not settle was the succession of the work. Donald Alexander, thirty-one years his father's junior and still unconfirmed as operational heir, spent the week after the reading in the Stephen Avenue rooms, learning which of the two ledgers — cattle or petroleum — the house would be judged by. The Viscount, asked, declined to answer. The fence was finished. Who would ride it was another season's business.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" t="n">
+        <v>2</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Clocks resumed from last recorded anchor</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>turn</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>2026-09-06 03:38:14</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Every house resumes at personal 1867, its last recorded anchor — a founding grant for the founding generation, an accession reset for the rest. The personal years elapsed between that anchor and the rebuild were not recovered and are not estimated. From here, clocks move only when a turn moves them: explicitly, house by house, or by a sync on a direct shared event.</t>
         </is>
       </c>
     </row>
@@ -15516,7 +15550,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>discharged</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Phase 9c A1-A2: split scenarios, add the engine tables
Moves the reconstructed game under scenarios/legacy/ (seed/, turns/,
RECONSTRUCTION.md) and adds an empty scenarios/new/ for the autoplay
game, with scenario.json manifests and scenarios/current.txt naming the
one hoc.db is built from. hoc/scenario.py resolves every path from it,
so load_seed, rebuild, the exporters and the tests no longer hard-code
data/seed or turns/; `python -m hoc scenario list|use` switches games and
the site's status strip names the active one.

rebuild.py replays whichever record the scenario has: turns/*.json for a
director-written game, seasons/NNNN.json for an engine-played one.

Schema gains the Phase 9c tables: house_stats, persons, objectives and
seasons, with 'kin' documented in relations.marker and era band ids in
climate.era_cohort. Every v1 table is untouched.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XTWKXtPrL9rvaUy4BKDKHi
</commit_message>
<xml_diff>
--- a/outputs/Riding_Tracker.xlsx
+++ b/outputs/Riding_Tracker.xlsx
@@ -7409,7 +7409,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see scenarios/legacy/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L2" t="n">
@@ -7467,7 +7467,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see scenarios/legacy/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L3" t="n">
@@ -7520,7 +7520,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see scenarios/legacy/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L4" t="n">
@@ -7573,7 +7573,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see scenarios/legacy/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L5" t="n">
@@ -7626,7 +7626,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see scenarios/legacy/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L6" t="n">
@@ -7679,7 +7679,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see scenarios/legacy/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L7" t="n">
@@ -7732,7 +7732,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see scenarios/legacy/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L8" t="n">
@@ -7790,7 +7790,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see scenarios/legacy/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L9" t="n">
@@ -7833,7 +7833,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see scenarios/legacy/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L10" t="n">
@@ -7886,7 +7886,7 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see scenarios/legacy/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L11" t="n">
@@ -7939,7 +7939,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see scenarios/legacy/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L12" t="n">
@@ -7997,7 +7997,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see scenarios/legacy/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L13" t="n">
@@ -8055,7 +8055,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see scenarios/legacy/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L14" t="n">
@@ -8103,7 +8103,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see scenarios/legacy/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L15" t="n">
@@ -8151,7 +8151,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see scenarios/legacy/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L16" t="n">
@@ -8204,7 +8204,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see scenarios/legacy/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L17" t="n">
@@ -8262,7 +8262,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see scenarios/legacy/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L18" t="n">
@@ -8310,7 +8310,7 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see scenarios/legacy/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L19" t="n">
@@ -8368,7 +8368,7 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see scenarios/legacy/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L20" t="n">
@@ -8421,7 +8421,7 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see scenarios/legacy/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L21" t="n">
@@ -8479,7 +8479,7 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see scenarios/legacy/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L22" t="n">
@@ -8532,7 +8532,7 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see scenarios/legacy/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L23" t="n">
@@ -8580,7 +8580,7 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see scenarios/legacy/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L24" t="n">
@@ -8633,7 +8633,7 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see scenarios/legacy/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L25" t="n">
@@ -8691,7 +8691,7 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see scenarios/legacy/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L26" t="n">
@@ -8749,7 +8749,7 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see scenarios/legacy/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L27" t="n">
@@ -8807,7 +8807,7 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see scenarios/legacy/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L28" t="n">
@@ -8860,7 +8860,7 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see scenarios/legacy/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L29" t="n">
@@ -8913,7 +8913,7 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see scenarios/legacy/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L30" t="n">
@@ -8971,7 +8971,7 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see scenarios/legacy/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L31" t="n">
@@ -9024,7 +9024,7 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see scenarios/legacy/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L32" t="n">
@@ -9082,7 +9082,7 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see scenarios/legacy/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L33" t="n">
@@ -9135,7 +9135,7 @@
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see scenarios/legacy/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L34" t="n">
@@ -9188,7 +9188,7 @@
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see scenarios/legacy/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L35" t="n">
@@ -9221,7 +9221,7 @@
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see docs/RECONSTRUCTION.md</t>
+          <t>resumed from last recorded anchor (personal 1867 at founding or at accession reset); intervening personal years not recovered — see scenarios/legacy/RECONSTRUCTION.md</t>
         </is>
       </c>
       <c r="L36" t="n">
@@ -14252,7 +14252,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-09-06T03:38:14+00:00</t>
+          <t>2026-09-06T19:51:35+00:00</t>
         </is>
       </c>
     </row>
@@ -14282,7 +14282,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-09-06T03:38:14+00:00</t>
+          <t>2026-09-06T19:51:35+00:00</t>
         </is>
       </c>
     </row>
@@ -14312,7 +14312,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-09-06T03:38:14+00:00</t>
+          <t>2026-09-06T19:51:35+00:00</t>
         </is>
       </c>
     </row>
@@ -14342,7 +14342,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-09-06T03:38:14+00:00</t>
+          <t>2026-09-06T19:51:35+00:00</t>
         </is>
       </c>
     </row>
@@ -14372,7 +14372,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-09-06T03:38:14+00:00</t>
+          <t>2026-09-06T19:51:35+00:00</t>
         </is>
       </c>
     </row>
@@ -14402,7 +14402,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-09-06T03:38:14+00:00</t>
+          <t>2026-09-06T19:51:35+00:00</t>
         </is>
       </c>
     </row>
@@ -14432,7 +14432,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-09-06T03:38:14+00:00</t>
+          <t>2026-09-06T19:51:35+00:00</t>
         </is>
       </c>
     </row>
@@ -14462,7 +14462,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-09-06T03:38:14+00:00</t>
+          <t>2026-09-06T19:51:35+00:00</t>
         </is>
       </c>
     </row>
@@ -14492,7 +14492,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-09-06T03:38:14+00:00</t>
+          <t>2026-09-06T19:51:35+00:00</t>
         </is>
       </c>
     </row>
@@ -14522,7 +14522,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-09-06T03:38:14+00:00</t>
+          <t>2026-09-06T19:51:35+00:00</t>
         </is>
       </c>
     </row>
@@ -14552,7 +14552,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-09-06T03:38:14+00:00</t>
+          <t>2026-09-06T19:51:35+00:00</t>
         </is>
       </c>
     </row>
@@ -14582,7 +14582,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-09-06T03:38:14+00:00</t>
+          <t>2026-09-06T19:51:35+00:00</t>
         </is>
       </c>
     </row>
@@ -14612,7 +14612,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-09-06T03:38:14+00:00</t>
+          <t>2026-09-06T19:51:35+00:00</t>
         </is>
       </c>
     </row>
@@ -14642,7 +14642,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-09-06T03:38:14+00:00</t>
+          <t>2026-09-06T19:51:35+00:00</t>
         </is>
       </c>
     </row>
@@ -14672,7 +14672,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026-09-06T03:38:14+00:00</t>
+          <t>2026-09-06T19:51:35+00:00</t>
         </is>
       </c>
     </row>
@@ -14702,7 +14702,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026-09-06T03:38:14+00:00</t>
+          <t>2026-09-06T19:51:35+00:00</t>
         </is>
       </c>
     </row>
@@ -14732,7 +14732,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026-09-06T03:38:14+00:00</t>
+          <t>2026-09-06T19:51:35+00:00</t>
         </is>
       </c>
     </row>
@@ -14762,7 +14762,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2026-09-06T03:38:14+00:00</t>
+          <t>2026-09-06T19:51:35+00:00</t>
         </is>
       </c>
     </row>
@@ -14792,7 +14792,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>2026-09-06T03:38:14+00:00</t>
+          <t>2026-09-06T19:51:35+00:00</t>
         </is>
       </c>
     </row>
@@ -14822,7 +14822,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>2026-09-06T03:38:14+00:00</t>
+          <t>2026-09-06T19:51:35+00:00</t>
         </is>
       </c>
     </row>
@@ -14852,7 +14852,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>2026-09-06T03:38:14+00:00</t>
+          <t>2026-09-06T19:51:35+00:00</t>
         </is>
       </c>
     </row>
@@ -14882,7 +14882,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>2026-09-06T03:38:14+00:00</t>
+          <t>2026-09-06T19:51:35+00:00</t>
         </is>
       </c>
     </row>
@@ -14912,7 +14912,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>2026-09-06T03:38:14+00:00</t>
+          <t>2026-09-06T19:51:35+00:00</t>
         </is>
       </c>
     </row>
@@ -14942,7 +14942,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>2026-09-06T03:38:14+00:00</t>
+          <t>2026-09-06T19:51:35+00:00</t>
         </is>
       </c>
     </row>
@@ -14972,7 +14972,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>2026-09-06T03:38:14+00:00</t>
+          <t>2026-09-06T19:51:35+00:00</t>
         </is>
       </c>
     </row>
@@ -15002,7 +15002,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>2026-09-06T03:38:14+00:00</t>
+          <t>2026-09-06T19:51:35+00:00</t>
         </is>
       </c>
     </row>
@@ -15032,7 +15032,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>2026-09-06T03:38:14+00:00</t>
+          <t>2026-09-06T19:51:35+00:00</t>
         </is>
       </c>
     </row>
@@ -15062,7 +15062,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>2026-09-06T03:38:14+00:00</t>
+          <t>2026-09-06T19:51:35+00:00</t>
         </is>
       </c>
     </row>
@@ -15092,7 +15092,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>2026-09-06T03:38:14+00:00</t>
+          <t>2026-09-06T19:51:35+00:00</t>
         </is>
       </c>
     </row>
@@ -15122,7 +15122,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>2026-09-06T03:38:14+00:00</t>
+          <t>2026-09-06T19:51:35+00:00</t>
         </is>
       </c>
     </row>
@@ -15152,7 +15152,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>2026-09-06T03:38:14+00:00</t>
+          <t>2026-09-06T19:51:35+00:00</t>
         </is>
       </c>
     </row>
@@ -15182,7 +15182,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>2026-09-06T03:38:14+00:00</t>
+          <t>2026-09-06T19:51:35+00:00</t>
         </is>
       </c>
     </row>
@@ -15212,7 +15212,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>2026-09-06T03:38:14+00:00</t>
+          <t>2026-09-06T19:51:35+00:00</t>
         </is>
       </c>
     </row>
@@ -15242,7 +15242,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>2026-09-06T03:38:14+00:00</t>
+          <t>2026-09-06T19:51:35+00:00</t>
         </is>
       </c>
     </row>
@@ -15272,7 +15272,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>2026-09-06T03:38:14+00:00</t>
+          <t>2026-09-06T19:51:35+00:00</t>
         </is>
       </c>
     </row>
@@ -15302,7 +15302,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>2026-09-06T03:38:14+00:00</t>
+          <t>2026-09-06T19:51:35+00:00</t>
         </is>
       </c>
     </row>
@@ -15332,7 +15332,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>2026-09-06T03:38:14+00:00</t>
+          <t>2026-09-06T19:51:35+00:00</t>
         </is>
       </c>
     </row>
@@ -15362,7 +15362,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>2026-09-06T03:38:14+00:00</t>
+          <t>2026-09-06T19:51:35+00:00</t>
         </is>
       </c>
     </row>
@@ -15392,7 +15392,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>2026-09-06T03:38:14+00:00</t>
+          <t>2026-09-06T19:51:35+00:00</t>
         </is>
       </c>
     </row>
@@ -15422,7 +15422,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>2026-09-06T03:38:14+00:00</t>
+          <t>2026-09-06T19:51:35+00:00</t>
         </is>
       </c>
     </row>
@@ -15455,7 +15455,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>2026-09-06 03:38:14</t>
+          <t>2026-09-06 19:51:35</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -15494,7 +15494,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>2026-09-06 03:38:14</t>
+          <t>2026-09-06 19:51:35</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">

</xml_diff>

<commit_message>
Phase 9d PART C: the Archive
scripts/build_archive.py builds the legacy scenario into a temporary
database and renders it through the same exporter as the live game, into
outputs/site/archive/ with a banner and the nav pointing back out rather
than deeper in. It is not a copy kept on the side: it is rebuilt on
every export, from `python -m hoc export` and from scripts/rebuild.py
alike, so a change to the site is a change to both and the two can never
drift. The temporary database is thrown away; hoc.db is never touched.

The archive carries no scrubber (a director's game has no seasons to
scrub) and every page offers a way back at whatever depth it sits.
"Archive" joins the main nav and about.html explains what it is.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XTWKXtPrL9rvaUy4BKDKHi
</commit_message>
<xml_diff>
--- a/outputs/Riding_Tracker.xlsx
+++ b/outputs/Riding_Tracker.xlsx
@@ -14252,7 +14252,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-09-06T21:03:47+00:00</t>
+          <t>2026-09-06T21:05:03+00:00</t>
         </is>
       </c>
     </row>
@@ -14282,7 +14282,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-09-06T21:03:47+00:00</t>
+          <t>2026-09-06T21:05:03+00:00</t>
         </is>
       </c>
     </row>
@@ -14312,7 +14312,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-09-06T21:03:47+00:00</t>
+          <t>2026-09-06T21:05:03+00:00</t>
         </is>
       </c>
     </row>
@@ -14342,7 +14342,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-09-06T21:03:47+00:00</t>
+          <t>2026-09-06T21:05:03+00:00</t>
         </is>
       </c>
     </row>
@@ -14372,7 +14372,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-09-06T21:03:47+00:00</t>
+          <t>2026-09-06T21:05:03+00:00</t>
         </is>
       </c>
     </row>
@@ -14402,7 +14402,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-09-06T21:03:47+00:00</t>
+          <t>2026-09-06T21:05:03+00:00</t>
         </is>
       </c>
     </row>
@@ -14432,7 +14432,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-09-06T21:03:47+00:00</t>
+          <t>2026-09-06T21:05:03+00:00</t>
         </is>
       </c>
     </row>
@@ -14462,7 +14462,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-09-06T21:03:47+00:00</t>
+          <t>2026-09-06T21:05:03+00:00</t>
         </is>
       </c>
     </row>
@@ -14492,7 +14492,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-09-06T21:03:47+00:00</t>
+          <t>2026-09-06T21:05:03+00:00</t>
         </is>
       </c>
     </row>
@@ -14522,7 +14522,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-09-06T21:03:47+00:00</t>
+          <t>2026-09-06T21:05:03+00:00</t>
         </is>
       </c>
     </row>
@@ -14552,7 +14552,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-09-06T21:03:47+00:00</t>
+          <t>2026-09-06T21:05:03+00:00</t>
         </is>
       </c>
     </row>
@@ -14582,7 +14582,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-09-06T21:03:47+00:00</t>
+          <t>2026-09-06T21:05:03+00:00</t>
         </is>
       </c>
     </row>
@@ -14612,7 +14612,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-09-06T21:03:47+00:00</t>
+          <t>2026-09-06T21:05:03+00:00</t>
         </is>
       </c>
     </row>
@@ -14642,7 +14642,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-09-06T21:03:47+00:00</t>
+          <t>2026-09-06T21:05:03+00:00</t>
         </is>
       </c>
     </row>
@@ -14672,7 +14672,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026-09-06T21:03:47+00:00</t>
+          <t>2026-09-06T21:05:03+00:00</t>
         </is>
       </c>
     </row>
@@ -14702,7 +14702,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026-09-06T21:03:47+00:00</t>
+          <t>2026-09-06T21:05:03+00:00</t>
         </is>
       </c>
     </row>
@@ -14732,7 +14732,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026-09-06T21:03:47+00:00</t>
+          <t>2026-09-06T21:05:03+00:00</t>
         </is>
       </c>
     </row>
@@ -14762,7 +14762,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2026-09-06T21:03:47+00:00</t>
+          <t>2026-09-06T21:05:03+00:00</t>
         </is>
       </c>
     </row>
@@ -14792,7 +14792,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>2026-09-06T21:03:47+00:00</t>
+          <t>2026-09-06T21:05:03+00:00</t>
         </is>
       </c>
     </row>
@@ -14822,7 +14822,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>2026-09-06T21:03:47+00:00</t>
+          <t>2026-09-06T21:05:03+00:00</t>
         </is>
       </c>
     </row>
@@ -14852,7 +14852,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>2026-09-06T21:03:47+00:00</t>
+          <t>2026-09-06T21:05:03+00:00</t>
         </is>
       </c>
     </row>
@@ -14882,7 +14882,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>2026-09-06T21:03:47+00:00</t>
+          <t>2026-09-06T21:05:03+00:00</t>
         </is>
       </c>
     </row>
@@ -14912,7 +14912,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>2026-09-06T21:03:47+00:00</t>
+          <t>2026-09-06T21:05:03+00:00</t>
         </is>
       </c>
     </row>
@@ -14942,7 +14942,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>2026-09-06T21:03:47+00:00</t>
+          <t>2026-09-06T21:05:03+00:00</t>
         </is>
       </c>
     </row>
@@ -14972,7 +14972,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>2026-09-06T21:03:47+00:00</t>
+          <t>2026-09-06T21:05:03+00:00</t>
         </is>
       </c>
     </row>
@@ -15002,7 +15002,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>2026-09-06T21:03:47+00:00</t>
+          <t>2026-09-06T21:05:03+00:00</t>
         </is>
       </c>
     </row>
@@ -15032,7 +15032,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>2026-09-06T21:03:47+00:00</t>
+          <t>2026-09-06T21:05:03+00:00</t>
         </is>
       </c>
     </row>
@@ -15062,7 +15062,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>2026-09-06T21:03:47+00:00</t>
+          <t>2026-09-06T21:05:03+00:00</t>
         </is>
       </c>
     </row>
@@ -15092,7 +15092,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>2026-09-06T21:03:47+00:00</t>
+          <t>2026-09-06T21:05:03+00:00</t>
         </is>
       </c>
     </row>
@@ -15122,7 +15122,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>2026-09-06T21:03:47+00:00</t>
+          <t>2026-09-06T21:05:03+00:00</t>
         </is>
       </c>
     </row>
@@ -15152,7 +15152,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>2026-09-06T21:03:47+00:00</t>
+          <t>2026-09-06T21:05:03+00:00</t>
         </is>
       </c>
     </row>
@@ -15182,7 +15182,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>2026-09-06T21:03:47+00:00</t>
+          <t>2026-09-06T21:05:03+00:00</t>
         </is>
       </c>
     </row>
@@ -15212,7 +15212,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>2026-09-06T21:03:47+00:00</t>
+          <t>2026-09-06T21:05:03+00:00</t>
         </is>
       </c>
     </row>
@@ -15242,7 +15242,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>2026-09-06T21:03:47+00:00</t>
+          <t>2026-09-06T21:05:03+00:00</t>
         </is>
       </c>
     </row>
@@ -15272,7 +15272,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>2026-09-06T21:03:47+00:00</t>
+          <t>2026-09-06T21:05:03+00:00</t>
         </is>
       </c>
     </row>
@@ -15302,7 +15302,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>2026-09-06T21:03:47+00:00</t>
+          <t>2026-09-06T21:05:03+00:00</t>
         </is>
       </c>
     </row>
@@ -15332,7 +15332,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>2026-09-06T21:03:47+00:00</t>
+          <t>2026-09-06T21:05:03+00:00</t>
         </is>
       </c>
     </row>
@@ -15362,7 +15362,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>2026-09-06T21:03:47+00:00</t>
+          <t>2026-09-06T21:05:03+00:00</t>
         </is>
       </c>
     </row>
@@ -15392,7 +15392,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>2026-09-06T21:03:47+00:00</t>
+          <t>2026-09-06T21:05:03+00:00</t>
         </is>
       </c>
     </row>
@@ -15422,7 +15422,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>2026-09-06T21:03:47+00:00</t>
+          <t>2026-09-06T21:05:03+00:00</t>
         </is>
       </c>
     </row>
@@ -15455,7 +15455,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>2026-09-06 21:03:47</t>
+          <t>2026-09-06 21:05:03</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -15494,7 +15494,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>2026-09-06 21:03:47</t>
+          <t>2026-09-06 21:05:03</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">

</xml_diff>

<commit_message>
run: seasons 2–6 (2 houses, 3 ridings)
</commit_message>
<xml_diff>
--- a/outputs/Riding_Tracker.xlsx
+++ b/outputs/Riding_Tracker.xlsx
@@ -38,7 +38,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -55,6 +55,16 @@
         <fgColor rgb="00c63939"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002f8989"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0058c6c6"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -68,13 +78,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -440,16 +452,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="47" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
   </cols>
@@ -533,6 +545,76 @@
         </is>
       </c>
       <c r="I2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Cashin</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Leeds—Grenville—Thousand Islands—Rideau Lakes</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Baron</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Baron Cashin of Dundas</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>#c63939</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Cox</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Mississauga East—Cooksville</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Viscount</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Viscount Cox of Temagami</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>#2f8989</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
         <v>1</v>
       </c>
     </row>
@@ -577,13 +659,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
@@ -688,7 +770,7 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>1867</v>
+        <v>1872</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -696,6 +778,49 @@
         </is>
       </c>
       <c r="L2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Cox</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Viscount</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Viscount Cox of Temagami</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>#2f8989</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>#58c6c6</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>1868</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>founded season 5</t>
+        </is>
+      </c>
+      <c r="L3" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1013,11 +1138,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1031,6 +1157,11 @@
           <t>Cashin</t>
         </is>
       </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Cox</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1039,6 +1170,16 @@
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Cox</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1051,14 +1192,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="21" customWidth="1" min="8" max="8"/>
@@ -1149,6 +1290,206 @@
       <c r="I2" t="inlineStr">
         <is>
           <t>Season 1 · Baron Cashin of Dundas is created, seated at Kingston and the Islands.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>societal</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>confederation</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Red River Resistance</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Cashin</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>engine</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2026-09-07 12:36:59</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Season 3 · Baron Cashin of Dundas meets Red River Resistance and resists.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>societal</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>confederation</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Confederation Extension (Manitoba Act)</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Cashin</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>engine</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2026-09-07 12:36:59</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Season 4 · Baron Cashin of Dundas meets Confederation Extension (Manitoba Act) and resists.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>expansion</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>confederation</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Baron Cashin of Dundas takes Leeds—Grenville—Thousand Islands—Rideau Lakes</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Cashin</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>engine</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2026-09-07 12:36:59</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Season 4 · Baron Cashin of Dundas takes Leeds—Grenville—Thousand Islands—Rideau Lakes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>societal</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>confederation</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>British Columbia Joins; Treaty 1 Signed</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Cashin</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>engine</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2026-09-07 12:36:59</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Season 5 · Baron Cashin of Dundas meets British Columbia Joins; Treaty 1 Signed and resists.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>founding</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>confederation</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Viscount Cox of Temagami founded</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Cox</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>engine</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2026-09-07 12:36:59</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Season 5 · Viscount Cox of Temagami is created, seated at Mississauga East—Cooksville.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Live world: restart at rules 0.7 on seed 1867, seat Kingston and the Islands
Phase 10-1 PART A4. Every draw in the game changed with the new generator, so
seasons 1-6 as played under rules 0.6 could no longer be replayed from their
own record: scripts/rebuild.py would have produced a different map from the
same seed, which is the one thing the record must never do.

The six seasons are discarded and the world re-founded on the same seed and
the same seat. scenarios/new/scenario.json records the restart and why.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XTWKXtPrL9rvaUy4BKDKHi
</commit_message>
<xml_diff>
--- a/outputs/Riding_Tracker.xlsx
+++ b/outputs/Riding_Tracker.xlsx
@@ -38,7 +38,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -47,22 +47,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00772222"/>
+        <fgColor rgb="00673232"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00c63939"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="002f8989"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="0058c6c6"/>
+        <fgColor rgb="00ac5353"/>
       </patternFill>
     </fill>
   </fills>
@@ -78,15 +68,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -452,16 +440,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="47" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
   </cols>
@@ -516,7 +504,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Cashin</t>
+          <t>Elliott</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -536,85 +524,15 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Baron Cashin of Dundas</t>
+          <t>Baron Elliott of Glengarry</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>#772222</t>
+          <t>#673232</t>
         </is>
       </c>
       <c r="I2" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Cashin</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Leeds—Grenville—Thousand Islands—Rideau Lakes</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Baron</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Baron Cashin of Dundas</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>#c63939</t>
-        </is>
-      </c>
-      <c r="I3" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Cox</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Mississauga East—Cooksville</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Viscount</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Viscount Cox of Temagami</t>
-        </is>
-      </c>
-      <c r="H4" s="4" t="inlineStr">
-        <is>
-          <t>#2f8989</t>
-        </is>
-      </c>
-      <c r="I4" t="n">
         <v>1</v>
       </c>
     </row>
@@ -659,13 +577,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
@@ -741,7 +659,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Cashin</t>
+          <t>Elliott</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -756,21 +674,21 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Baron Cashin of Dundas</t>
+          <t>Baron Elliott of Glengarry</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>#772222</t>
+          <t>#673232</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>#c63939</t>
+          <t>#ac5353</t>
         </is>
       </c>
       <c r="J2" t="n">
-        <v>1872</v>
+        <v>1867</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -778,49 +696,6 @@
         </is>
       </c>
       <c r="L2" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Cox</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Viscount</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Viscount Cox of Temagami</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>#2f8989</t>
-        </is>
-      </c>
-      <c r="F3" s="5" t="inlineStr">
-        <is>
-          <t>#58c6c6</t>
-        </is>
-      </c>
-      <c r="J3" t="n">
-        <v>1868</v>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>founded season 5</t>
-        </is>
-      </c>
-      <c r="L3" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1138,12 +1013,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1154,32 +1028,17 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Cashin</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Cox</t>
+          <t>Elliott</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Cashin</t>
+          <t>Elliott</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Cox</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1192,14 +1051,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="21" customWidth="1" min="8" max="8"/>
@@ -1269,12 +1128,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Baron Cashin of Dundas founded</t>
+          <t>Baron Elliott of Glengarry founded</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Cashin</t>
+          <t>Elliott</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -1284,212 +1143,12 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-09-06 21:50:20</t>
+          <t>2026-09-07 12:54:42</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Season 1 · Baron Cashin of Dundas is created, seated at Kingston and the Islands.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>2</v>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>societal</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>confederation</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Red River Resistance</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Cashin</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>engine</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>2026-09-07 12:36:59</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Season 3 · Baron Cashin of Dundas meets Red River Resistance and resists.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>3</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>societal</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>confederation</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Confederation Extension (Manitoba Act)</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Cashin</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>engine</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>2026-09-07 12:36:59</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Season 4 · Baron Cashin of Dundas meets Confederation Extension (Manitoba Act) and resists.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>4</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>expansion</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>confederation</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Baron Cashin of Dundas takes Leeds—Grenville—Thousand Islands—Rideau Lakes</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Cashin</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>engine</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>2026-09-07 12:36:59</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>Season 4 · Baron Cashin of Dundas takes Leeds—Grenville—Thousand Islands—Rideau Lakes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>5</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>societal</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>confederation</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>British Columbia Joins; Treaty 1 Signed</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Cashin</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>engine</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>2026-09-07 12:36:59</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Season 5 · Baron Cashin of Dundas meets British Columbia Joins; Treaty 1 Signed and resists.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>6</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>founding</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>confederation</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Viscount Cox of Temagami founded</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Cox</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>engine</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>2026-09-07 12:36:59</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>Season 5 · Viscount Cox of Temagami is created, seated at Mississauga East—Cooksville.</t>
+          <t>Season 1 · Baron Elliott of Glengarry is created, seated at Kingston and the Islands.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Referee: verified seasons 2–3; exported
</commit_message>
<xml_diff>
--- a/outputs/Riding_Tracker.xlsx
+++ b/outputs/Riding_Tracker.xlsx
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>1867</v>
+        <v>1869</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -1051,7 +1051,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1143,12 +1143,52 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-09-07 12:54:42</t>
+          <t>2026-09-07 15:58:14</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
           <t>Season 1 · Baron Elliott of Glengarry is created, seated at Kingston and the Islands.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>societal</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>confederation</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Red River Resistance</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Elliott</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>engine</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2026-09-07 15:58:14</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Season 3 · Baron Elliott of Glengarry meets Red River Resistance and exploits.</t>
         </is>
       </c>
     </row>

</xml_diff>